<commit_message>
Se agregan documentos faltantes a la carpeta de CFD y se realiza la reunión de avance del proyecto. Se actualiza la especificación del proyecto y se toman notas en la documentación de registro de reuniones.
</commit_message>
<xml_diff>
--- a/05_Diseño_Mecánico/Matriz_Decision_Arquitectura_Banco.xlsx
+++ b/05_Diseño_Mecánico/Matriz_Decision_Arquitectura_Banco.xlsx
@@ -1,14 +1,31 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="20" documentId="11_F4E11FFFDB0C346B1EE0404D5600A798F8EC3839" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{104D210B-E24C-47A9-8957-466A558E7EE9}"/>
+  <bookViews>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Instrucciones" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="Torque - Motor de Carga" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="Angulo - Sensor" state="visible" r:id="rId6"/>
+    <sheet name="Instrucciones" sheetId="1" r:id="rId1"/>
+    <sheet name="Torque - Motor de Carga" sheetId="2" r:id="rId2"/>
+    <sheet name="Angulo - Sensor" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="171027"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -207,59 +224,68 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="10" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
       <sz val="14"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <i/>
+      <sz val="10"/>
       <color rgb="FF555555"/>
-      <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <i/>
+      <sz val="9"/>
       <color rgb="FF555555"/>
-      <sz val="9"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
+      <sz val="11"/>
       <color rgb="FF0000FF"/>
-      <sz val="11"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
+      <sz val="11"/>
       <color rgb="FF000000"/>
-      <sz val="11"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <i/>
       <sz val="11"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="5">
@@ -314,21 +340,11 @@
   </cellStyleXfs>
   <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="bottom"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -338,42 +354,26 @@
     <xf numFmtId="10" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="10" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="bottom"/>
-    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="10" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="bottom"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="bottom" wrapText="1"/>
+      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="bottom"/>
+      <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="10" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="2" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="bottom"/>
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="10" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="bottom"/>
-    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -712,99 +712,99 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:A15"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="96.71428571428571" customWidth="1"/>
-    <col min="2" max="24" width="13.571428571428571" customWidth="1"/>
+    <col min="1" max="1" width="96.7109375" customWidth="1"/>
+    <col min="2" max="24" width="13.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="17.25" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>11</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:G20"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="42.142857142857146" customWidth="1"/>
+    <col min="1" max="1" width="83.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10" customWidth="1"/>
     <col min="3" max="6" width="24" customWidth="1"/>
-    <col min="7" max="7" width="42.142857142857146" customWidth="1"/>
-    <col min="8" max="24" width="13.571428571428571" customWidth="1"/>
+    <col min="7" max="7" width="42.140625" customWidth="1"/>
+    <col min="8" max="24" width="13.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="17.25" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>12</v>
       </c>
@@ -815,7 +815,7 @@
       <c r="F1" s="3"/>
       <c r="G1" s="3"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>13</v>
       </c>
@@ -826,7 +826,7 @@
       <c r="F2" s="3"/>
       <c r="G2" s="3"/>
     </row>
-    <row r="3" ht="26.25" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="6"/>
       <c r="B3" s="6"/>
       <c r="C3" s="6"/>
@@ -835,7 +835,7 @@
       <c r="F3" s="6"/>
       <c r="G3" s="3"/>
     </row>
-    <row r="4" ht="39" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" ht="39" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
         <v>14</v>
       </c>
@@ -858,7 +858,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="5" ht="39" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" ht="72" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
         <v>21</v>
       </c>
@@ -881,7 +881,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="6" ht="39" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" ht="57.75" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
         <v>23</v>
       </c>
@@ -904,7 +904,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="7" ht="39" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" ht="57.75" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
         <v>25</v>
       </c>
@@ -927,7 +927,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="8" ht="51.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" ht="72" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
         <v>27</v>
       </c>
@@ -950,7 +950,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="9" ht="51.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" ht="100.5" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
         <v>29</v>
       </c>
@@ -973,7 +973,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="10" ht="51.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" ht="72" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
         <v>31</v>
       </c>
@@ -996,7 +996,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="11" ht="51.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" ht="86.25" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>33</v>
       </c>
@@ -1019,7 +1019,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" ht="100.5" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
         <v>35</v>
       </c>
@@ -1042,7 +1042,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" ht="86.25" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
         <v>37</v>
       </c>
@@ -1065,7 +1065,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" ht="114.75" x14ac:dyDescent="0.25">
       <c r="A14" s="9" t="s">
         <v>39</v>
       </c>
@@ -1088,7 +1088,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" ht="100.5" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
         <v>41</v>
       </c>
@@ -1111,7 +1111,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" ht="72" x14ac:dyDescent="0.25">
       <c r="A16" s="9" t="s">
         <v>43</v>
       </c>
@@ -1134,74 +1134,83 @@
         <v>44</v>
       </c>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="14" t="s">
         <v>45</v>
       </c>
       <c r="B17" s="15">
         <f>SUM(B5:B16)</f>
-      </c>
-    </row>
-    <row r="19" ht="15" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="16" t="s">
         <v>46</v>
       </c>
       <c r="B19" s="17"/>
       <c r="C19" s="18">
         <f>SUMPRODUCT(B5:B16,C5:C16)</f>
+        <v>4.1399999999999997</v>
       </c>
       <c r="D19" s="18">
         <f>SUMPRODUCT(B5:B16,D5:D16)</f>
+        <v>2.56</v>
       </c>
       <c r="E19" s="18">
         <f>SUMPRODUCT(B5:B16,E5:E16)</f>
+        <v>2.44</v>
       </c>
       <c r="F19" s="18">
         <f>SUMPRODUCT(B5:B16,F5:F16)</f>
-      </c>
-    </row>
-    <row r="20" ht="15" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2.2399999999999998</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="14" t="s">
         <v>47</v>
       </c>
       <c r="B20" s="17"/>
       <c r="C20" s="19">
         <f>RANK(C19,$C$19:$F$19)</f>
+        <v>1</v>
       </c>
       <c r="D20" s="19">
         <f>RANK(D19,$C$19:$F$19)</f>
+        <v>2</v>
       </c>
       <c r="E20" s="19">
         <f>RANK(E19,$C$19:$F$19)</f>
+        <v>3</v>
       </c>
       <c r="F20" s="19">
         <f>RANK(F19,$C$19:$F$19)</f>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:E13"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="42" customWidth="1"/>
+    <col min="1" max="1" width="52.140625" customWidth="1"/>
     <col min="2" max="2" width="10" customWidth="1"/>
     <col min="3" max="4" width="22" customWidth="1"/>
-    <col min="5" max="5" width="42.142857142857146" customWidth="1"/>
-    <col min="6" max="24" width="13.571428571428571" customWidth="1"/>
+    <col min="5" max="5" width="42.140625" customWidth="1"/>
+    <col min="6" max="24" width="13.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="17.25" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
         <v>14</v>
       </c>
@@ -1218,7 +1227,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" ht="39" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" ht="57.75" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>51</v>
       </c>
@@ -1235,7 +1244,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="5" ht="51.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" ht="57.75" x14ac:dyDescent="0.25">
       <c r="A5" s="20" t="s">
         <v>53</v>
       </c>
@@ -1252,7 +1261,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="6" ht="51.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" ht="72" x14ac:dyDescent="0.25">
       <c r="A6" s="20" t="s">
         <v>55</v>
       </c>
@@ -1269,7 +1278,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="7" ht="39" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" ht="57.75" x14ac:dyDescent="0.25">
       <c r="A7" s="20" t="s">
         <v>57</v>
       </c>
@@ -1286,7 +1295,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="8" ht="51.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="20" t="s">
         <v>59</v>
       </c>
@@ -1303,7 +1312,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="9" ht="51.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" ht="57.75" x14ac:dyDescent="0.25">
       <c r="A9" s="20" t="s">
         <v>61</v>
       </c>
@@ -1320,40 +1329,45 @@
         <v>62</v>
       </c>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
         <v>45</v>
       </c>
       <c r="B10" s="15">
         <f>SUM(B4:B9)</f>
-      </c>
-    </row>
-    <row r="12" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+        <v>1.0000000000000002</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="16" t="s">
         <v>46</v>
       </c>
       <c r="B12" s="17"/>
       <c r="C12" s="18">
         <f>SUMPRODUCT(B4:B9,C4:C9)</f>
+        <v>3.5</v>
       </c>
       <c r="D12" s="18">
         <f>SUMPRODUCT(B4:B9,D4:D9)</f>
-      </c>
-    </row>
-    <row r="13" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
         <v>47</v>
       </c>
       <c r="B13" s="17"/>
       <c r="C13" s="19">
         <f>RANK(C12,$C$12:$D$12)</f>
+        <v>2</v>
       </c>
       <c r="D13" s="19">
         <f>RANK(D12,$C$12:$D$12)</f>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>